<commit_message>
S12: pivot 演習1 to spreadsheet fill-in worksheet
Replace "先に紙で設計" with a pre-built 情報設計 spreadsheet template
where the 考え方・判断基準 column is pre-filled by the instructor and
students fill the あなたの答え column while consulting Gemini. Adds a
Gemini相談ログ sheet to capture the consultation pattern.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MLnStsm4YQNeGye3rc2BGH
</commit_message>
<xml_diff>
--- a/lecture_pptx/session12_assets/お金情報配信_デモデータ.xlsx
+++ b/lecture_pptx/session12_assets/お金情報配信_デモデータ.xlsx
@@ -10,6 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="情報設計" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="情報源マスター" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="配信予約" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gemini相談ログ" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -36,12 +37,12 @@
     <font>
       <name val="Yu Gothic UI"/>
       <b val="1"/>
+      <color rgb="001F3A5F"/>
       <sz val="11"/>
     </font>
     <font>
       <name val="Yu Gothic UI"/>
-      <b val="1"/>
-      <color rgb="001F3A5F"/>
+      <color rgb="001A1A1A"/>
       <sz val="11"/>
     </font>
     <font>
@@ -49,7 +50,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -63,12 +64,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F4F6F9"/>
+        <fgColor rgb="00E8A33D"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E8A33D"/>
+        <fgColor rgb="00C76B7A"/>
       </patternFill>
     </fill>
     <fill>
@@ -78,12 +79,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F3A5F"/>
+        <fgColor rgb="00F4F6F9"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00C76B7A"/>
+        <fgColor rgb="00FCEEF0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F3A5F"/>
       </patternFill>
     </fill>
     <fill>
@@ -118,37 +124,52 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -515,198 +536,271 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:D14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="60" customWidth="1" min="2" max="2"/>
-    <col width="35" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="48" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28" customHeight="1">
+    <row r="1" ht="42" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>項目</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>設計内容</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>なぜそう決めたか</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="50" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>考え方・判断基準
+(先にここを読む)</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>あなたの答え
+(ここを埋める)</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>例
+(参考、そのまま写さない)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="78" customHeight="1">
+      <c r="A2" s="5" t="inlineStr">
         <is>
           <t>ターゲット読者像</t>
         </is>
       </c>
-      <c r="B2" s="3" t="inlineStr">
-        <is>
-          <t>お金の知識に自信がない30〜50代。会社員/自営業/主婦を含む。難しい言葉が並ぶと即離脱するので、平易な説明を最優先。</t>
-        </is>
-      </c>
-      <c r="C2" s="3" t="inlineStr">
-        <is>
-          <t>離脱しないため</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="50" customHeight="1">
-      <c r="A3" s="4" t="inlineStr">
+      <c r="B2" s="6" t="inlineStr">
+        <is>
+          <t>誰に配信するか決めないと、AIに"分かりやすい"を判定してもらえない。年齢/職業/お金の知識レベル/読むシーン(通勤中?)まで具体化する。</t>
+        </is>
+      </c>
+      <c r="C2" s="7" t="inlineStr"/>
+      <c r="D2" s="6" t="inlineStr">
+        <is>
+          <t>お金の知識に自信がない30〜50代の会社員。通勤中スマホでチラ見。</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="78" customHeight="1">
+      <c r="A3" s="8" t="inlineStr">
         <is>
           <t>カテゴリ①</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr">
-        <is>
-          <t>助成金・補助金 (中小企業向け, 個人向け)</t>
-        </is>
-      </c>
-      <c r="C3" s="5" t="inlineStr">
-        <is>
-          <t>"知らずに損した" 感が最も大きい領域</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="50" customHeight="1">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="B3" s="9" t="inlineStr">
+        <is>
+          <t>毎回テーマがブレると"この人は何の人?"になる。最初に4カテゴリ程度に絞ると、AIが偏らず選べる。</t>
+        </is>
+      </c>
+      <c r="C3" s="7" t="inlineStr"/>
+      <c r="D3" s="9" t="inlineStr">
+        <is>
+          <t>助成金・補助金</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="78" customHeight="1">
+      <c r="A4" s="5" t="inlineStr">
         <is>
           <t>カテゴリ②</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>税金・節税対策 (確定申告, iDeCo, NISA関連)</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>最新の税制改正に敏感な層が多い</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="50" customHeight="1">
-      <c r="A5" s="4" t="inlineStr">
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>同上。全カテゴリの合計配信本数が同程度になる想定で決める。</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr"/>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>税金・節税</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="78" customHeight="1">
+      <c r="A5" s="8" t="inlineStr">
         <is>
           <t>カテゴリ③</t>
         </is>
       </c>
-      <c r="B5" s="5" t="inlineStr">
-        <is>
-          <t>株・為替の "考え方" (市況解説は避ける)</t>
-        </is>
-      </c>
-      <c r="C5" s="5" t="inlineStr">
-        <is>
-          <t>個別助言NG。基礎知識のみ配信</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="50" customHeight="1">
-      <c r="A6" s="2" t="inlineStr">
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>同上。株為替は"市況予想"ではなく"考え方"や"用語解説"に留める。</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr"/>
+      <c r="D5" s="9" t="inlineStr">
+        <is>
+          <t>株・為替(考え方のみ、予想NG)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="78" customHeight="1">
+      <c r="A6" s="5" t="inlineStr">
         <is>
           <t>カテゴリ④</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>お金の豆知識 (公的手当, 制度の使い方)</t>
-        </is>
-      </c>
-      <c r="C6" s="3" t="inlineStr">
-        <is>
-          <t>生活に直結、シェアされやすい</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="50" customHeight="1">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>同上。生活に近い豆知識はシェアされやすい。</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr"/>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>お金の豆知識(年金/手当/制度)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="78" customHeight="1">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>情報源(ホワイトリスト)</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="inlineStr">
+        <is>
+          <t>AIが個人ブログ/アフィリを引かないよう、"許可サイトのリスト"を渡す。公的機関を軸に、迷ったら金融庁で代替できるようにする。</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr"/>
+      <c r="D7" s="9" t="inlineStr">
+        <is>
+          <t>国税庁 / 金融庁 / 中小企業庁 / 厚労省 / 経産省 / 日銀 / 統計局 / 年金機構 / 政府広報 / J-Net21</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="78" customHeight="1">
+      <c r="A8" s="5" t="inlineStr">
         <is>
           <t>タイトルの型</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr">
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>LINE のトーク一覧で"開くか閉じるか"を決めるのはタイトル。文字数を先に決めておくとAIの生成が安定する。</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr"/>
+      <c r="D8" s="6" t="inlineStr">
         <is>
           <t>20文字以内、絵文字は末尾1つまで</t>
         </is>
       </c>
-      <c r="C7" s="5" t="inlineStr">
-        <is>
-          <t>LINE のトーク一覧で埋もれない</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="50" customHeight="1">
-      <c r="A8" s="2" t="inlineStr">
+    </row>
+    <row r="9" ht="78" customHeight="1">
+      <c r="A9" s="8" t="inlineStr">
         <is>
           <t>本文の型</t>
         </is>
       </c>
-      <c r="B8" s="3" t="inlineStr">
-        <is>
-          <t>300文字以内、3〜5行で改行、末尾に出典URL</t>
-        </is>
-      </c>
-      <c r="C8" s="3" t="inlineStr">
-        <is>
-          <t>スマホで1画面完結</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="50" customHeight="1">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>出典URLルール</t>
-        </is>
-      </c>
-      <c r="B9" s="5" t="inlineStr">
-        <is>
-          <t>本文末に必ず添付、ホワイトリスト外はNG</t>
-        </is>
-      </c>
-      <c r="C9" s="5" t="inlineStr">
-        <is>
-          <t>信頼性と誤情報防止</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="50" customHeight="1">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>個別助言の禁止</t>
-        </is>
-      </c>
-      <c r="B10" s="3" t="inlineStr">
-        <is>
-          <t>税務相談・投資判断はしない、"詳しくは専門家/公式サイトへ" で締める</t>
-        </is>
-      </c>
-      <c r="C10" s="3" t="inlineStr">
-        <is>
-          <t>金融商品取引法/税理士法対策</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="50" customHeight="1">
-      <c r="A11" s="4" t="inlineStr">
+      <c r="B9" s="9" t="inlineStr">
+        <is>
+          <t>スマホで1画面で完結する量にする。改行の入れ方も指定するとリズムが揃う。</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="inlineStr"/>
+      <c r="D9" s="9" t="inlineStr">
+        <is>
+          <t>300字以内 / 3〜5行改行 / 平易な表現 / 末尾に出典URL</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="78" customHeight="1">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>出典URLの扱い</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>出典なしは"信頼できない情報"扱いされる。必ず本文末に添付、ドメインはホワイトリスト内のみ。</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="inlineStr"/>
+      <c r="D10" s="6" t="inlineStr">
+        <is>
+          <t>本文末に必須。ホワイトリスト外のURLは配信しない</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="78" customHeight="1">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>やらないこと(禁止事項)</t>
+        </is>
+      </c>
+      <c r="B11" s="9" t="inlineStr">
+        <is>
+          <t>個別助言は法令違反リスク。売り込みも信頼を落とす。"やらない範囲"を明文化しておくとAIが暴走しない。</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="inlineStr"/>
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t>個別税務相談 / 個別投資助言 / 特定商品推奨 / 売り込み文言</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="78" customHeight="1">
+      <c r="A12" s="5" t="inlineStr">
         <is>
           <t>配信頻度</t>
         </is>
       </c>
-      <c r="B11" s="5" t="inlineStr">
-        <is>
-          <t>週1〜2回、朝9時 (デモは手動)</t>
-        </is>
-      </c>
-      <c r="C11" s="5" t="inlineStr">
-        <is>
-          <t>無料枠200通/月を意識</t>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>週2以上は継続できない人が多い。無理せず"3ヶ月続く量"を決める。</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="inlineStr"/>
+      <c r="D12" s="6" t="inlineStr">
+        <is>
+          <t>週1回(まずは)、慣れたら週2に</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="78" customHeight="1">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>配信時間帯</t>
+        </is>
+      </c>
+      <c r="B13" s="9" t="inlineStr">
+        <is>
+          <t>ターゲットが読める時間帯。通勤中/昼休み/夜が候補。</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="inlineStr"/>
+      <c r="D13" s="9" t="inlineStr">
+        <is>
+          <t>平日 朝9時前(通勤で開く時間)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="78" customHeight="1">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>OK/NGの判定基準</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>AI生成をそのまま配信しない。何を見てOKにするか、事前に基準を決めておくと迷わない。</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="inlineStr"/>
+      <c r="D14" s="6" t="inlineStr">
+        <is>
+          <t>出典が本当にホワイトリスト内 / 数字が正しい / 個別助言なし / トーンが自分の3軸に合う</t>
         </is>
       </c>
     </row>
@@ -721,13 +815,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
     <col width="25" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="50" customWidth="1" min="4" max="4"/>
+    <col width="45" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -736,241 +831,256 @@
           <t>機関名</t>
         </is>
       </c>
-      <c r="B1" s="6" t="inlineStr">
+      <c r="B1" s="2" t="inlineStr">
         <is>
           <t>ドメイン</t>
         </is>
       </c>
-      <c r="C1" s="7" t="inlineStr">
+      <c r="C1" s="4" t="inlineStr">
         <is>
           <t>主なカテゴリ</t>
         </is>
       </c>
-      <c r="D1" s="8" t="inlineStr">
+      <c r="D1" s="10" t="inlineStr">
         <is>
           <t>メモ</t>
         </is>
       </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>採用/不採用</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="42" customHeight="1">
-      <c r="A2" s="3" t="inlineStr">
+      <c r="A2" s="11" t="inlineStr">
         <is>
           <t>国税庁</t>
         </is>
       </c>
-      <c r="B2" s="3" t="inlineStr">
+      <c r="B2" s="11" t="inlineStr">
         <is>
           <t>nta.go.jp</t>
         </is>
       </c>
-      <c r="C2" s="3" t="inlineStr">
+      <c r="C2" s="11" t="inlineStr">
         <is>
           <t>税金</t>
         </is>
       </c>
-      <c r="D2" s="3" t="inlineStr">
+      <c r="D2" s="11" t="inlineStr">
         <is>
           <t>すべての税金情報の一次ソース。個別相談は税理士会へ誘導。</t>
         </is>
       </c>
+      <c r="E2" s="12" t="inlineStr"/>
     </row>
     <row r="3" ht="42" customHeight="1">
-      <c r="A3" s="5" t="inlineStr">
+      <c r="A3" s="13" t="inlineStr">
         <is>
           <t>金融庁</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr">
+      <c r="B3" s="13" t="inlineStr">
         <is>
           <t>fsa.go.jp</t>
         </is>
       </c>
-      <c r="C3" s="5" t="inlineStr">
+      <c r="C3" s="13" t="inlineStr">
         <is>
           <t>株為替/豆知識</t>
         </is>
       </c>
-      <c r="D3" s="5" t="inlineStr">
+      <c r="D3" s="13" t="inlineStr">
         <is>
           <t>金融教育コンテンツが充実。NISA/iDeCo等の基礎解説。</t>
         </is>
       </c>
+      <c r="E3" s="12" t="inlineStr"/>
     </row>
     <row r="4" ht="42" customHeight="1">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="11" t="inlineStr">
         <is>
           <t>中小企業庁</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="11" t="inlineStr">
         <is>
           <t>chusho.meti.go.jp</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="11" t="inlineStr">
         <is>
           <t>助成金</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="11" t="inlineStr">
         <is>
           <t>中小・小規模事業者向け補助金・支援策の入り口。</t>
         </is>
       </c>
+      <c r="E4" s="12" t="inlineStr"/>
     </row>
     <row r="5" ht="42" customHeight="1">
-      <c r="A5" s="5" t="inlineStr">
+      <c r="A5" s="13" t="inlineStr">
         <is>
           <t>J-Net21 (中小機構)</t>
         </is>
       </c>
-      <c r="B5" s="5" t="inlineStr">
+      <c r="B5" s="13" t="inlineStr">
         <is>
           <t>j-net21.smrj.go.jp</t>
         </is>
       </c>
-      <c r="C5" s="5" t="inlineStr">
+      <c r="C5" s="13" t="inlineStr">
         <is>
           <t>助成金</t>
         </is>
       </c>
-      <c r="D5" s="5" t="inlineStr">
+      <c r="D5" s="13" t="inlineStr">
         <is>
           <t>補助金検索・事例が豊富、一般人が読みやすい。</t>
         </is>
       </c>
+      <c r="E5" s="12" t="inlineStr"/>
     </row>
     <row r="6" ht="42" customHeight="1">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="A6" s="11" t="inlineStr">
         <is>
           <t>厚生労働省</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" s="11" t="inlineStr">
         <is>
           <t>mhlw.go.jp</t>
         </is>
       </c>
-      <c r="C6" s="3" t="inlineStr">
+      <c r="C6" s="11" t="inlineStr">
         <is>
           <t>助成金/豆知識</t>
         </is>
       </c>
-      <c r="D6" s="3" t="inlineStr">
+      <c r="D6" s="11" t="inlineStr">
         <is>
           <t>雇用調整助成金/教育訓練給付など働く人向け。</t>
         </is>
       </c>
+      <c r="E6" s="12" t="inlineStr"/>
     </row>
     <row r="7" ht="42" customHeight="1">
-      <c r="A7" s="5" t="inlineStr">
+      <c r="A7" s="13" t="inlineStr">
         <is>
           <t>経済産業省</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr">
+      <c r="B7" s="13" t="inlineStr">
         <is>
           <t>meti.go.jp</t>
         </is>
       </c>
-      <c r="C7" s="5" t="inlineStr">
+      <c r="C7" s="13" t="inlineStr">
         <is>
           <t>助成金</t>
         </is>
       </c>
-      <c r="D7" s="5" t="inlineStr">
+      <c r="D7" s="13" t="inlineStr">
         <is>
           <t>ものづくり補助金・IT導入補助金など事業者向け。</t>
         </is>
       </c>
+      <c r="E7" s="12" t="inlineStr"/>
     </row>
     <row r="8" ht="42" customHeight="1">
-      <c r="A8" s="3" t="inlineStr">
+      <c r="A8" s="11" t="inlineStr">
         <is>
           <t>日本銀行</t>
         </is>
       </c>
-      <c r="B8" s="3" t="inlineStr">
+      <c r="B8" s="11" t="inlineStr">
         <is>
           <t>boj.or.jp</t>
         </is>
       </c>
-      <c r="C8" s="3" t="inlineStr">
+      <c r="C8" s="11" t="inlineStr">
         <is>
           <t>株為替</t>
         </is>
       </c>
-      <c r="D8" s="3" t="inlineStr">
+      <c r="D8" s="11" t="inlineStr">
         <is>
           <t>金融政策・為替の一次情報。速報より背景解説向き。</t>
         </is>
       </c>
+      <c r="E8" s="12" t="inlineStr"/>
     </row>
     <row r="9" ht="42" customHeight="1">
-      <c r="A9" s="5" t="inlineStr">
+      <c r="A9" s="13" t="inlineStr">
         <is>
           <t>総務省 統計局</t>
         </is>
       </c>
-      <c r="B9" s="5" t="inlineStr">
+      <c r="B9" s="13" t="inlineStr">
         <is>
           <t>stat.go.jp</t>
         </is>
       </c>
-      <c r="C9" s="5" t="inlineStr">
+      <c r="C9" s="13" t="inlineStr">
         <is>
           <t>豆知識</t>
         </is>
       </c>
-      <c r="D9" s="5" t="inlineStr">
+      <c r="D9" s="13" t="inlineStr">
         <is>
           <t>家計調査・物価指数など、生活に近い統計データ。</t>
         </is>
       </c>
+      <c r="E9" s="12" t="inlineStr"/>
     </row>
     <row r="10" ht="42" customHeight="1">
-      <c r="A10" s="3" t="inlineStr">
+      <c r="A10" s="11" t="inlineStr">
         <is>
           <t>日本年金機構</t>
         </is>
       </c>
-      <c r="B10" s="3" t="inlineStr">
+      <c r="B10" s="11" t="inlineStr">
         <is>
           <t>nenkin.go.jp</t>
         </is>
       </c>
-      <c r="C10" s="3" t="inlineStr">
+      <c r="C10" s="11" t="inlineStr">
         <is>
           <t>豆知識</t>
         </is>
       </c>
-      <c r="D10" s="3" t="inlineStr">
+      <c r="D10" s="11" t="inlineStr">
         <is>
           <t>年金制度の公式解説、老後資金の基礎データ。</t>
         </is>
       </c>
+      <c r="E10" s="12" t="inlineStr"/>
     </row>
     <row r="11" ht="42" customHeight="1">
-      <c r="A11" s="5" t="inlineStr">
+      <c r="A11" s="13" t="inlineStr">
         <is>
           <t>政府広報オンライン</t>
         </is>
       </c>
-      <c r="B11" s="5" t="inlineStr">
+      <c r="B11" s="13" t="inlineStr">
         <is>
           <t>gov-online.go.jp</t>
         </is>
       </c>
-      <c r="C11" s="5" t="inlineStr">
+      <c r="C11" s="13" t="inlineStr">
         <is>
           <t>豆知識</t>
         </is>
       </c>
-      <c r="D11" s="5" t="inlineStr">
+      <c r="D11" s="13" t="inlineStr">
         <is>
           <t>一般人向けに噛み砕いた政府施策の紹介。</t>
         </is>
       </c>
+      <c r="E11" s="12" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -990,7 +1100,7 @@
     <col width="26" customWidth="1" min="2" max="2"/>
     <col width="60" customWidth="1" min="3" max="3"/>
     <col width="36" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
   </cols>
@@ -1001,12 +1111,12 @@
           <t>生成日時</t>
         </is>
       </c>
-      <c r="B1" s="6" t="inlineStr">
+      <c r="B1" s="2" t="inlineStr">
         <is>
           <t>タイトル</t>
         </is>
       </c>
-      <c r="C1" s="7" t="inlineStr">
+      <c r="C1" s="4" t="inlineStr">
         <is>
           <t>本文</t>
         </is>
@@ -1016,108 +1126,172 @@
           <t>出典URL</t>
         </is>
       </c>
-      <c r="E1" s="8" t="inlineStr">
+      <c r="E1" s="10" t="inlineStr">
         <is>
           <t>カテゴリ</t>
         </is>
       </c>
-      <c r="F1" s="9" t="inlineStr">
+      <c r="F1" s="3" t="inlineStr">
         <is>
           <t>OK/NG</t>
         </is>
       </c>
-      <c r="G1" s="10" t="inlineStr">
+      <c r="G1" s="14" t="inlineStr">
         <is>
           <t>配信済み日時</t>
         </is>
       </c>
     </row>
     <row r="2" ht="56" customHeight="1">
-      <c r="A2" s="3" t="inlineStr">
+      <c r="A2" s="11" t="inlineStr">
         <is>
           <t>2026/07/03 09:00</t>
         </is>
       </c>
-      <c r="B2" s="3" t="inlineStr">
+      <c r="B2" s="11" t="inlineStr">
         <is>
           <t>iDeCo改正で節税枠拡大 💰</t>
         </is>
       </c>
-      <c r="C2" s="3" t="inlineStr">
+      <c r="C2" s="11" t="inlineStr">
         <is>
           <t>2024年12月からiDeCoの拠出限度額が引き上げられ、より多くの人が節税と老後資金づくりを両立しやすくなりました。会社員は月2.3万円まで拠出可能に。所得税・住民税が軽くなる仕組みです。</t>
         </is>
       </c>
-      <c r="D2" s="3" t="inlineStr">
+      <c r="D2" s="11" t="inlineStr">
         <is>
           <t>https://www.fsa.go.jp/ordinary/annai.html</t>
         </is>
       </c>
-      <c r="E2" s="3" t="inlineStr">
-        <is>
-          <t>税金</t>
-        </is>
-      </c>
-      <c r="F2" s="3" t="inlineStr"/>
-      <c r="G2" s="3" t="inlineStr"/>
+      <c r="E2" s="11" t="inlineStr">
+        <is>
+          <t>税金・節税</t>
+        </is>
+      </c>
+      <c r="F2" s="11" t="inlineStr"/>
+      <c r="G2" s="11" t="inlineStr"/>
     </row>
     <row r="3" ht="56" customHeight="1">
-      <c r="A3" s="5" t="inlineStr">
+      <c r="A3" s="13" t="inlineStr">
         <is>
           <t>2026/07/03 09:00</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr">
+      <c r="B3" s="13" t="inlineStr">
         <is>
           <t>IT導入補助金2026 申請開始 💡</t>
         </is>
       </c>
-      <c r="C3" s="5" t="inlineStr">
+      <c r="C3" s="13" t="inlineStr">
         <is>
           <t>中小企業がITツール導入時の費用を最大450万円まで支援する「IT導入補助金2026」の公募が始まりました。会計ソフトやEC構築など幅広く対象。申請期限や書類は公式サイトで確認を。</t>
         </is>
       </c>
-      <c r="D3" s="5" t="inlineStr">
+      <c r="D3" s="13" t="inlineStr">
         <is>
           <t>https://www.chusho.meti.go.jp/</t>
         </is>
       </c>
-      <c r="E3" s="5" t="inlineStr">
-        <is>
-          <t>助成金</t>
-        </is>
-      </c>
-      <c r="F3" s="5" t="inlineStr"/>
-      <c r="G3" s="5" t="inlineStr"/>
+      <c r="E3" s="13" t="inlineStr">
+        <is>
+          <t>助成金・補助金</t>
+        </is>
+      </c>
+      <c r="F3" s="13" t="inlineStr"/>
+      <c r="G3" s="13" t="inlineStr"/>
     </row>
     <row r="4" ht="56" customHeight="1">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="11" t="inlineStr">
         <is>
           <t>2026/07/03 09:00</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>為替の "実質" って何？ 📊</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="B4" s="11" t="inlineStr">
+        <is>
+          <t>為替の "実質" って何? 📊</t>
+        </is>
+      </c>
+      <c r="C4" s="11" t="inlineStr">
         <is>
           <t>為替ニュースで見る「実質実効為替レート」は、他の通貨と比べた円の総合的な強さを表す指標です。名目レートと違い、物価変動も加味されるため、暮らしへの影響を測るのに使えます。</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="11" t="inlineStr">
         <is>
           <t>https://www.boj.or.jp/</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
-        <is>
-          <t>株為替</t>
-        </is>
-      </c>
-      <c r="F4" s="3" t="inlineStr"/>
-      <c r="G4" s="3" t="inlineStr"/>
+      <c r="E4" s="11" t="inlineStr">
+        <is>
+          <t>株・為替</t>
+        </is>
+      </c>
+      <c r="F4" s="11" t="inlineStr"/>
+      <c r="G4" s="11" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="45" customWidth="1" min="3" max="3"/>
+    <col width="45" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>日時</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>どの項目について</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>Geminiへの質問</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>自分の結論(スプシに書いた内容)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="56" customHeight="1">
+      <c r="A2" s="15" t="inlineStr">
+        <is>
+          <t>2026/07/03 10:15</t>
+        </is>
+      </c>
+      <c r="B2" s="15" t="inlineStr">
+        <is>
+          <t>配信頻度</t>
+        </is>
+      </c>
+      <c r="C2" s="15" t="inlineStr">
+        <is>
+          <t>週1と週2どっちが継続しやすい?私は業務で忙しいです。</t>
+        </is>
+      </c>
+      <c r="D2" s="15" t="inlineStr">
+        <is>
+          <t>週1回 木曜朝に決めた(まず3ヶ月続けて、余裕あれば週2に)</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
S12: add 情報設計_記入例 sheet + purge paper-based work references
- Add "情報設計_記入例" sheet: fully filled reference sheet (保険営業
  プランナー想定) so students see a completed design before filling
  their own. Green C-column = 記入見本, extra D-column = 判断理由.
- S12 ex1 target/situation now points students at the 記入例 sheet
  first for orientation, then back to 情報設計 to fill in their own.
- Remove "紙 or スプシで" / "紙で設計" / "紙に書く" phrasing from S11
  walkthrough, S12 slides, and S12 README.
- Add lecture_pptx/CLAUDE.md: codify no-paper-work rule + spreadsheet
  template pattern (テンプレ + 記入例 + 相談ログ の3点セット) for all
  future workshop design.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MLnStsm4YQNeGye3rc2BGH
</commit_message>
<xml_diff>
--- a/lecture_pptx/session12_assets/お金情報配信_デモデータ.xlsx
+++ b/lecture_pptx/session12_assets/お金情報配信_デモデータ.xlsx
@@ -8,9 +8,10 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="情報設計" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="情報源マスター" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="配信予約" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gemini相談ログ" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="情報設計_記入例" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="情報源マスター" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="配信予約" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gemini相談ログ" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -47,10 +48,16 @@
     </font>
     <font>
       <name val="Yu Gothic UI"/>
+      <b val="1"/>
+      <color rgb="001F3A5F"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Yu Gothic UI"/>
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="12">
     <fill>
       <patternFill/>
     </fill>
@@ -89,6 +96,16 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00FFF7E0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E6F4EA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="001F3A5F"/>
       </patternFill>
     </fill>
@@ -98,7 +115,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -120,11 +137,55 @@
         <color rgb="00D7DCE3"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00D7DCE3"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00D7DCE3"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D7DCE3"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00D7DCE3"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D7DCE3"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00D7DCE3"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D7DCE3"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D7DCE3"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -153,22 +214,30 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -815,6 +884,352 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:D15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
+    <col width="46" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="72" customHeight="1">
+      <c r="A1" s="10" t="inlineStr">
+        <is>
+          <t>■ この見本の使い方
+これは 保険営業プランナー(30-50代の家計相談中心)が「情報設計」テンプレを 実際に埋めたらこうなる、という完成見本です。
+「あなたの答え」列を "そのままコピペ" せずに、骨格の参考として眺めてから、
+「情報設計」シートに戻って自分の運用に合わせて書き直してください。</t>
+        </is>
+      </c>
+      <c r="B1" s="11" t="n"/>
+      <c r="C1" s="11" t="n"/>
+      <c r="D1" s="12" t="n"/>
+    </row>
+    <row r="2" ht="42" customHeight="1">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>項目</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>考え方・判断基準</t>
+        </is>
+      </c>
+      <c r="C2" s="1" t="inlineStr">
+        <is>
+          <t>あなたの答え
+(記入見本)</t>
+        </is>
+      </c>
+      <c r="D2" s="4" t="inlineStr">
+        <is>
+          <t>判断理由
+(なぜこう決めたか)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="90" customHeight="1">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>ターゲット読者像</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>誰に配信するか決めないと、AIに"分かりやすい"を判定してもらえない。年齢/職業/お金の知識レベル/読むシーン(通勤中?)まで具体化する。</t>
+        </is>
+      </c>
+      <c r="C3" s="13" t="inlineStr">
+        <is>
+          <t>既契約者+相談検討中の30〜50代 会社員/共働き家庭。お金の話は苦手意識ありで、通勤電車と昼休みにLINEを開く。</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="inlineStr">
+        <is>
+          <t>既存顧客の年齢層データから中央値40歳前後。共働きが多い層は"制度もの"の食いつきが良い。</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="90" customHeight="1">
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>カテゴリ①</t>
+        </is>
+      </c>
+      <c r="B4" s="9" t="inlineStr">
+        <is>
+          <t>毎回テーマがブレると"この人は何の人?"になる。最初に4カテゴリ程度に絞ると、AIが偏らず選べる。</t>
+        </is>
+      </c>
+      <c r="C4" s="13" t="inlineStr">
+        <is>
+          <t>税金・節税(iDeCo/ふるさと納税/確定申告)</t>
+        </is>
+      </c>
+      <c r="D4" s="9" t="inlineStr">
+        <is>
+          <t>相談上位テーマ。年末調整の時期に強い。</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="90" customHeight="1">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>カテゴリ②</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>同上。全カテゴリの合計配信本数が同程度になる想定で決める。</t>
+        </is>
+      </c>
+      <c r="C5" s="13" t="inlineStr">
+        <is>
+          <t>手当・給付(児童手当/傷病手当金/雇用保険)</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>共働き層に刺さる。相談化しやすい実利ネタ。</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="90" customHeight="1">
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>カテゴリ③</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>同上。株為替は"市況予想"ではなく"考え方"や"用語解説"に留める。</t>
+        </is>
+      </c>
+      <c r="C6" s="13" t="inlineStr">
+        <is>
+          <t>お金のリテラシー(用語解説/よくある誤解)</t>
+        </is>
+      </c>
+      <c r="D6" s="9" t="inlineStr">
+        <is>
+          <t>"予想"を避けるためあえて解説枠。金融庁の教育コンテンツを軸に。</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="90" customHeight="1">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>カテゴリ④</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>同上。生活に近い豆知識はシェアされやすい。</t>
+        </is>
+      </c>
+      <c r="C7" s="13" t="inlineStr">
+        <is>
+          <t>暮らしの制度豆知識(年金/医療費/公的サービス)</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>既契約者のリピート接点。家族に転送されやすい。</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="90" customHeight="1">
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>情報源(ホワイトリスト)</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>AIが個人ブログ/アフィリを引かないよう、"許可サイトのリスト"を渡す。公的機関を軸に、迷ったら金融庁で代替できるようにする。</t>
+        </is>
+      </c>
+      <c r="C8" s="13" t="inlineStr">
+        <is>
+          <t>国税庁 / 金融庁 / 厚労省 / 日本年金機構 / 政府広報オンライン / 総務省統計局 / 中小企業庁 / J-Net21</t>
+        </is>
+      </c>
+      <c r="D8" s="9" t="inlineStr">
+        <is>
+          <t>10サイトのうち"日銀・経産省"は自分の運用と遠いので落とした。予想系を避けるため日銀は除外。</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="90" customHeight="1">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>タイトルの型</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>LINE のトーク一覧で"開くか閉じるか"を決めるのはタイトル。文字数を先に決めておくとAIの生成が安定する。</t>
+        </is>
+      </c>
+      <c r="C9" s="13" t="inlineStr">
+        <is>
+          <t>18文字以内 / 絵文字は先頭に1つ / 数字を必ず1つ含める</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>スマホ通知プレビューが約19字。「数字」は開封率が上がる(iDeCo改正〇円UP的な)。</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="90" customHeight="1">
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>本文の型</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>スマホで1画面で完結する量にする。改行の入れ方も指定するとリズムが揃う。</t>
+        </is>
+      </c>
+      <c r="C10" s="13" t="inlineStr">
+        <is>
+          <t>250字以内 / 3行ごとに空行 / 語尾は"です・ます" / 最終行は「詳しくは↓」+ 出典URL</t>
+        </is>
+      </c>
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>短めが読了率高い。語尾はキャラを固定(硬すぎず砕けすぎず)。</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="90" customHeight="1">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>出典URLの扱い</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>出典なしは"信頼できない情報"扱いされる。必ず本文末に添付、ドメインはホワイトリスト内のみ。</t>
+        </is>
+      </c>
+      <c r="C11" s="13" t="inlineStr">
+        <is>
+          <t>本文末に必須、短縮URLは使わない、リンクプレビューが公的機関だと分かる状態を保つ。</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>短縮すると"詐欺?"と思われる。公的機関ドメインが見える方が信頼される。</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="90" customHeight="1">
+      <c r="A12" s="8" t="inlineStr">
+        <is>
+          <t>やらないこと(禁止事項)</t>
+        </is>
+      </c>
+      <c r="B12" s="9" t="inlineStr">
+        <is>
+          <t>個別助言は法令違反リスク。売り込みも信頼を落とす。"やらない範囲"を明文化しておくとAIが暴走しない。</t>
+        </is>
+      </c>
+      <c r="C12" s="13" t="inlineStr">
+        <is>
+          <t>個別税務相談 / 個別投資助言 / 特定保険商品の推奨 / 「今すぐ相談を」等の煽り / 期限を煽る表現</t>
+        </is>
+      </c>
+      <c r="D12" s="9" t="inlineStr">
+        <is>
+          <t>税理士法・保険業法・金商法で線引き必須。営業感を出すと配信ブロック率が上がる。</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="90" customHeight="1">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>配信頻度</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>週2以上は継続できない人が多い。無理せず"3ヶ月続く量"を決める。</t>
+        </is>
+      </c>
+      <c r="C13" s="13" t="inlineStr">
+        <is>
+          <t>週1回(木曜朝9時) / 月末に翌月4本の予告</t>
+        </is>
+      </c>
+      <c r="D13" s="6" t="inlineStr">
+        <is>
+          <t>朝一で受信→通勤で読了 の動線。木曜は面談枠が少ないので集計と配信を両立できる。</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="90" customHeight="1">
+      <c r="A14" s="8" t="inlineStr">
+        <is>
+          <t>配信時間帯</t>
+        </is>
+      </c>
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>ターゲットが読める時間帯。通勤中/昼休み/夜が候補。</t>
+        </is>
+      </c>
+      <c r="C14" s="13" t="inlineStr">
+        <is>
+          <t>木曜 8:45 (通勤ラッシュの前半)</t>
+        </is>
+      </c>
+      <c r="D14" s="9" t="inlineStr">
+        <is>
+          <t>ターゲット共働き層は8:30-9:00に電車移動が多い。</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="90" customHeight="1">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>OK/NGの判定基準</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>AI生成をそのまま配信しない。何を見てOKにするか、事前に基準を決めておくと迷わない。</t>
+        </is>
+      </c>
+      <c r="C15" s="13" t="inlineStr">
+        <is>
+          <t>① 出典URLがホワイトリスト内 / ② 数字が公式ソースと一致 / ③ 個別助言・煽りゼロ / ④ タイトル18字以内 / ⑤ 語尾トーン統一</t>
+        </is>
+      </c>
+      <c r="D15" s="6" t="inlineStr">
+        <is>
+          <t>この5点は毎回チェック。1つでも欠けたらNG、AIに書き直し依頼。</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:D1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -841,7 +1256,7 @@
           <t>主なカテゴリ</t>
         </is>
       </c>
-      <c r="D1" s="10" t="inlineStr">
+      <c r="D1" s="14" t="inlineStr">
         <is>
           <t>メモ</t>
         </is>
@@ -853,241 +1268,241 @@
       </c>
     </row>
     <row r="2" ht="42" customHeight="1">
-      <c r="A2" s="11" t="inlineStr">
+      <c r="A2" s="15" t="inlineStr">
         <is>
           <t>国税庁</t>
         </is>
       </c>
-      <c r="B2" s="11" t="inlineStr">
+      <c r="B2" s="15" t="inlineStr">
         <is>
           <t>nta.go.jp</t>
         </is>
       </c>
-      <c r="C2" s="11" t="inlineStr">
+      <c r="C2" s="15" t="inlineStr">
         <is>
           <t>税金</t>
         </is>
       </c>
-      <c r="D2" s="11" t="inlineStr">
+      <c r="D2" s="15" t="inlineStr">
         <is>
           <t>すべての税金情報の一次ソース。個別相談は税理士会へ誘導。</t>
         </is>
       </c>
-      <c r="E2" s="12" t="inlineStr"/>
+      <c r="E2" s="16" t="inlineStr"/>
     </row>
     <row r="3" ht="42" customHeight="1">
-      <c r="A3" s="13" t="inlineStr">
+      <c r="A3" s="17" t="inlineStr">
         <is>
           <t>金融庁</t>
         </is>
       </c>
-      <c r="B3" s="13" t="inlineStr">
+      <c r="B3" s="17" t="inlineStr">
         <is>
           <t>fsa.go.jp</t>
         </is>
       </c>
-      <c r="C3" s="13" t="inlineStr">
+      <c r="C3" s="17" t="inlineStr">
         <is>
           <t>株為替/豆知識</t>
         </is>
       </c>
-      <c r="D3" s="13" t="inlineStr">
+      <c r="D3" s="17" t="inlineStr">
         <is>
           <t>金融教育コンテンツが充実。NISA/iDeCo等の基礎解説。</t>
         </is>
       </c>
-      <c r="E3" s="12" t="inlineStr"/>
+      <c r="E3" s="16" t="inlineStr"/>
     </row>
     <row r="4" ht="42" customHeight="1">
-      <c r="A4" s="11" t="inlineStr">
+      <c r="A4" s="15" t="inlineStr">
         <is>
           <t>中小企業庁</t>
         </is>
       </c>
-      <c r="B4" s="11" t="inlineStr">
+      <c r="B4" s="15" t="inlineStr">
         <is>
           <t>chusho.meti.go.jp</t>
         </is>
       </c>
-      <c r="C4" s="11" t="inlineStr">
+      <c r="C4" s="15" t="inlineStr">
         <is>
           <t>助成金</t>
         </is>
       </c>
-      <c r="D4" s="11" t="inlineStr">
+      <c r="D4" s="15" t="inlineStr">
         <is>
           <t>中小・小規模事業者向け補助金・支援策の入り口。</t>
         </is>
       </c>
-      <c r="E4" s="12" t="inlineStr"/>
+      <c r="E4" s="16" t="inlineStr"/>
     </row>
     <row r="5" ht="42" customHeight="1">
-      <c r="A5" s="13" t="inlineStr">
+      <c r="A5" s="17" t="inlineStr">
         <is>
           <t>J-Net21 (中小機構)</t>
         </is>
       </c>
-      <c r="B5" s="13" t="inlineStr">
+      <c r="B5" s="17" t="inlineStr">
         <is>
           <t>j-net21.smrj.go.jp</t>
         </is>
       </c>
-      <c r="C5" s="13" t="inlineStr">
+      <c r="C5" s="17" t="inlineStr">
         <is>
           <t>助成金</t>
         </is>
       </c>
-      <c r="D5" s="13" t="inlineStr">
+      <c r="D5" s="17" t="inlineStr">
         <is>
           <t>補助金検索・事例が豊富、一般人が読みやすい。</t>
         </is>
       </c>
-      <c r="E5" s="12" t="inlineStr"/>
+      <c r="E5" s="16" t="inlineStr"/>
     </row>
     <row r="6" ht="42" customHeight="1">
-      <c r="A6" s="11" t="inlineStr">
+      <c r="A6" s="15" t="inlineStr">
         <is>
           <t>厚生労働省</t>
         </is>
       </c>
-      <c r="B6" s="11" t="inlineStr">
+      <c r="B6" s="15" t="inlineStr">
         <is>
           <t>mhlw.go.jp</t>
         </is>
       </c>
-      <c r="C6" s="11" t="inlineStr">
+      <c r="C6" s="15" t="inlineStr">
         <is>
           <t>助成金/豆知識</t>
         </is>
       </c>
-      <c r="D6" s="11" t="inlineStr">
+      <c r="D6" s="15" t="inlineStr">
         <is>
           <t>雇用調整助成金/教育訓練給付など働く人向け。</t>
         </is>
       </c>
-      <c r="E6" s="12" t="inlineStr"/>
+      <c r="E6" s="16" t="inlineStr"/>
     </row>
     <row r="7" ht="42" customHeight="1">
-      <c r="A7" s="13" t="inlineStr">
+      <c r="A7" s="17" t="inlineStr">
         <is>
           <t>経済産業省</t>
         </is>
       </c>
-      <c r="B7" s="13" t="inlineStr">
+      <c r="B7" s="17" t="inlineStr">
         <is>
           <t>meti.go.jp</t>
         </is>
       </c>
-      <c r="C7" s="13" t="inlineStr">
+      <c r="C7" s="17" t="inlineStr">
         <is>
           <t>助成金</t>
         </is>
       </c>
-      <c r="D7" s="13" t="inlineStr">
+      <c r="D7" s="17" t="inlineStr">
         <is>
           <t>ものづくり補助金・IT導入補助金など事業者向け。</t>
         </is>
       </c>
-      <c r="E7" s="12" t="inlineStr"/>
+      <c r="E7" s="16" t="inlineStr"/>
     </row>
     <row r="8" ht="42" customHeight="1">
-      <c r="A8" s="11" t="inlineStr">
+      <c r="A8" s="15" t="inlineStr">
         <is>
           <t>日本銀行</t>
         </is>
       </c>
-      <c r="B8" s="11" t="inlineStr">
+      <c r="B8" s="15" t="inlineStr">
         <is>
           <t>boj.or.jp</t>
         </is>
       </c>
-      <c r="C8" s="11" t="inlineStr">
+      <c r="C8" s="15" t="inlineStr">
         <is>
           <t>株為替</t>
         </is>
       </c>
-      <c r="D8" s="11" t="inlineStr">
+      <c r="D8" s="15" t="inlineStr">
         <is>
           <t>金融政策・為替の一次情報。速報より背景解説向き。</t>
         </is>
       </c>
-      <c r="E8" s="12" t="inlineStr"/>
+      <c r="E8" s="16" t="inlineStr"/>
     </row>
     <row r="9" ht="42" customHeight="1">
-      <c r="A9" s="13" t="inlineStr">
+      <c r="A9" s="17" t="inlineStr">
         <is>
           <t>総務省 統計局</t>
         </is>
       </c>
-      <c r="B9" s="13" t="inlineStr">
+      <c r="B9" s="17" t="inlineStr">
         <is>
           <t>stat.go.jp</t>
         </is>
       </c>
-      <c r="C9" s="13" t="inlineStr">
+      <c r="C9" s="17" t="inlineStr">
         <is>
           <t>豆知識</t>
         </is>
       </c>
-      <c r="D9" s="13" t="inlineStr">
+      <c r="D9" s="17" t="inlineStr">
         <is>
           <t>家計調査・物価指数など、生活に近い統計データ。</t>
         </is>
       </c>
-      <c r="E9" s="12" t="inlineStr"/>
+      <c r="E9" s="16" t="inlineStr"/>
     </row>
     <row r="10" ht="42" customHeight="1">
-      <c r="A10" s="11" t="inlineStr">
+      <c r="A10" s="15" t="inlineStr">
         <is>
           <t>日本年金機構</t>
         </is>
       </c>
-      <c r="B10" s="11" t="inlineStr">
+      <c r="B10" s="15" t="inlineStr">
         <is>
           <t>nenkin.go.jp</t>
         </is>
       </c>
-      <c r="C10" s="11" t="inlineStr">
+      <c r="C10" s="15" t="inlineStr">
         <is>
           <t>豆知識</t>
         </is>
       </c>
-      <c r="D10" s="11" t="inlineStr">
+      <c r="D10" s="15" t="inlineStr">
         <is>
           <t>年金制度の公式解説、老後資金の基礎データ。</t>
         </is>
       </c>
-      <c r="E10" s="12" t="inlineStr"/>
+      <c r="E10" s="16" t="inlineStr"/>
     </row>
     <row r="11" ht="42" customHeight="1">
-      <c r="A11" s="13" t="inlineStr">
+      <c r="A11" s="17" t="inlineStr">
         <is>
           <t>政府広報オンライン</t>
         </is>
       </c>
-      <c r="B11" s="13" t="inlineStr">
+      <c r="B11" s="17" t="inlineStr">
         <is>
           <t>gov-online.go.jp</t>
         </is>
       </c>
-      <c r="C11" s="13" t="inlineStr">
+      <c r="C11" s="17" t="inlineStr">
         <is>
           <t>豆知識</t>
         </is>
       </c>
-      <c r="D11" s="13" t="inlineStr">
+      <c r="D11" s="17" t="inlineStr">
         <is>
           <t>一般人向けに噛み砕いた政府施策の紹介。</t>
         </is>
       </c>
-      <c r="E11" s="12" t="inlineStr"/>
+      <c r="E11" s="16" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1126,7 +1541,7 @@
           <t>出典URL</t>
         </is>
       </c>
-      <c r="E1" s="10" t="inlineStr">
+      <c r="E1" s="14" t="inlineStr">
         <is>
           <t>カテゴリ</t>
         </is>
@@ -1136,105 +1551,105 @@
           <t>OK/NG</t>
         </is>
       </c>
-      <c r="G1" s="14" t="inlineStr">
+      <c r="G1" s="18" t="inlineStr">
         <is>
           <t>配信済み日時</t>
         </is>
       </c>
     </row>
     <row r="2" ht="56" customHeight="1">
-      <c r="A2" s="11" t="inlineStr">
+      <c r="A2" s="15" t="inlineStr">
         <is>
           <t>2026/07/03 09:00</t>
         </is>
       </c>
-      <c r="B2" s="11" t="inlineStr">
+      <c r="B2" s="15" t="inlineStr">
         <is>
           <t>iDeCo改正で節税枠拡大 💰</t>
         </is>
       </c>
-      <c r="C2" s="11" t="inlineStr">
+      <c r="C2" s="15" t="inlineStr">
         <is>
           <t>2024年12月からiDeCoの拠出限度額が引き上げられ、より多くの人が節税と老後資金づくりを両立しやすくなりました。会社員は月2.3万円まで拠出可能に。所得税・住民税が軽くなる仕組みです。</t>
         </is>
       </c>
-      <c r="D2" s="11" t="inlineStr">
+      <c r="D2" s="15" t="inlineStr">
         <is>
           <t>https://www.fsa.go.jp/ordinary/annai.html</t>
         </is>
       </c>
-      <c r="E2" s="11" t="inlineStr">
+      <c r="E2" s="15" t="inlineStr">
         <is>
           <t>税金・節税</t>
         </is>
       </c>
-      <c r="F2" s="11" t="inlineStr"/>
-      <c r="G2" s="11" t="inlineStr"/>
+      <c r="F2" s="15" t="inlineStr"/>
+      <c r="G2" s="15" t="inlineStr"/>
     </row>
     <row r="3" ht="56" customHeight="1">
-      <c r="A3" s="13" t="inlineStr">
+      <c r="A3" s="17" t="inlineStr">
         <is>
           <t>2026/07/03 09:00</t>
         </is>
       </c>
-      <c r="B3" s="13" t="inlineStr">
+      <c r="B3" s="17" t="inlineStr">
         <is>
           <t>IT導入補助金2026 申請開始 💡</t>
         </is>
       </c>
-      <c r="C3" s="13" t="inlineStr">
+      <c r="C3" s="17" t="inlineStr">
         <is>
           <t>中小企業がITツール導入時の費用を最大450万円まで支援する「IT導入補助金2026」の公募が始まりました。会計ソフトやEC構築など幅広く対象。申請期限や書類は公式サイトで確認を。</t>
         </is>
       </c>
-      <c r="D3" s="13" t="inlineStr">
+      <c r="D3" s="17" t="inlineStr">
         <is>
           <t>https://www.chusho.meti.go.jp/</t>
         </is>
       </c>
-      <c r="E3" s="13" t="inlineStr">
+      <c r="E3" s="17" t="inlineStr">
         <is>
           <t>助成金・補助金</t>
         </is>
       </c>
-      <c r="F3" s="13" t="inlineStr"/>
-      <c r="G3" s="13" t="inlineStr"/>
+      <c r="F3" s="17" t="inlineStr"/>
+      <c r="G3" s="17" t="inlineStr"/>
     </row>
     <row r="4" ht="56" customHeight="1">
-      <c r="A4" s="11" t="inlineStr">
+      <c r="A4" s="15" t="inlineStr">
         <is>
           <t>2026/07/03 09:00</t>
         </is>
       </c>
-      <c r="B4" s="11" t="inlineStr">
+      <c r="B4" s="15" t="inlineStr">
         <is>
           <t>為替の "実質" って何? 📊</t>
         </is>
       </c>
-      <c r="C4" s="11" t="inlineStr">
+      <c r="C4" s="15" t="inlineStr">
         <is>
           <t>為替ニュースで見る「実質実効為替レート」は、他の通貨と比べた円の総合的な強さを表す指標です。名目レートと違い、物価変動も加味されるため、暮らしへの影響を測るのに使えます。</t>
         </is>
       </c>
-      <c r="D4" s="11" t="inlineStr">
+      <c r="D4" s="15" t="inlineStr">
         <is>
           <t>https://www.boj.or.jp/</t>
         </is>
       </c>
-      <c r="E4" s="11" t="inlineStr">
+      <c r="E4" s="15" t="inlineStr">
         <is>
           <t>株・為替</t>
         </is>
       </c>
-      <c r="F4" s="11" t="inlineStr"/>
-      <c r="G4" s="11" t="inlineStr"/>
+      <c r="F4" s="15" t="inlineStr"/>
+      <c r="G4" s="15" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1272,22 +1687,22 @@
       </c>
     </row>
     <row r="2" ht="56" customHeight="1">
-      <c r="A2" s="15" t="inlineStr">
+      <c r="A2" s="19" t="inlineStr">
         <is>
           <t>2026/07/03 10:15</t>
         </is>
       </c>
-      <c r="B2" s="15" t="inlineStr">
+      <c r="B2" s="19" t="inlineStr">
         <is>
           <t>配信頻度</t>
         </is>
       </c>
-      <c r="C2" s="15" t="inlineStr">
+      <c r="C2" s="19" t="inlineStr">
         <is>
           <t>週1と週2どっちが継続しやすい?私は業務で忙しいです。</t>
         </is>
       </c>
-      <c r="D2" s="15" t="inlineStr">
+      <c r="D2" s="19" t="inlineStr">
         <is>
           <t>週1回 木曜朝に決めた(まず3ヶ月続けて、余裕あれば週2に)</t>
         </is>

</xml_diff>